<commit_message>
adding frontend tramites and oficinas
</commit_message>
<xml_diff>
--- a/backend/data/oficinas.xlsx
+++ b/backend/data/oficinas.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sebas\OneDrive\Documentos\TripleTen\guanajuato_chatbot\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/9a2c1a913e52701c/Documentos/TripleTen/guanajuato_chatbot/backend/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1909E5F7-01CA-4D39-BB30-8BCE1D6AD7D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{1909E5F7-01CA-4D39-BB30-8BCE1D6AD7D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8698CB86-5421-43B0-AB13-CF2C29B9AB2F}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{DD898DDE-4268-4E68-B508-281B6456CEB0}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="481" uniqueCount="191">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="482" uniqueCount="192">
   <si>
     <t>Abasolo</t>
   </si>
@@ -607,6 +607,9 @@
   </si>
   <si>
     <t>idOficina</t>
+  </si>
+  <si>
+    <t>xº</t>
   </si>
 </sst>
 </file>
@@ -1876,8 +1879,8 @@
       </c>
     </row>
     <row r="23" spans="1:11" ht="55.2" customHeight="1" thickBot="1">
-      <c r="A23">
-        <v>22</v>
+      <c r="A23" t="s">
+        <v>191</v>
       </c>
       <c r="B23" s="9" t="s">
         <v>89</v>

</xml_diff>